<commit_message>
feat(parser): add script to convert Excel sheet to JSON for conjunto_b_optim dataset
</commit_message>
<xml_diff>
--- a/evaluation/datasets/Diseño.xlsx
+++ b/evaluation/datasets/Diseño.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30224"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="449" documentId="11_9248B46DC1CBB2E3ED7FF6F9903E8C1851038383" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{22E5DB31-7E48-4E30-AA51-9D1A34D65A5B}"/>
+  <xr:revisionPtr revIDLastSave="466" documentId="11_9248B46DC1CBB2E3ED7FF6F9903E8C1851038383" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7E33A33E-D828-451E-B109-98C0D6F803A4}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cobertura del corpus" sheetId="1" r:id="rId1"/>
@@ -14,6 +14,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Dataset Conjunto A'!$B$5:$L$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Dataset Conjunto B'!$B$5:$F$5</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="487" uniqueCount="351">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="892" uniqueCount="591">
   <si>
     <t>Norma</t>
   </si>
@@ -1212,12 +1213,732 @@
   <si>
     <t>examen de egreso, terminación laboral</t>
   </si>
+  <si>
+    <t>B001</t>
+  </si>
+  <si>
+    <t>Empresa que quiere confirmar a quién le aplica la normativa de clasificación de riesgos.</t>
+  </si>
+  <si>
+    <t>¿A quién aplica el Decreto 768 de 2022?</t>
+  </si>
+  <si>
+    <t>B002</t>
+  </si>
+  <si>
+    <t>Empresa con dos sucursales que realizan actividades económicas distintas.</t>
+  </si>
+  <si>
+    <t>Si mis dos sedes tienen actividades diferentes, ¿pueden tener clases de riesgo distintas?</t>
+  </si>
+  <si>
+    <t>B003</t>
+  </si>
+  <si>
+    <t>Empresa cuya actividad económica no aparece en la tabla CIIU del decreto.</t>
+  </si>
+  <si>
+    <t>¿Qué pasa si mi actividad económica no está en la tabla de clasificación de riesgos?</t>
+  </si>
+  <si>
+    <t>B004</t>
+  </si>
+  <si>
+    <t>Empresa a la que le cambió la clase de riesgo tras una actualización de la tabla.</t>
+  </si>
+  <si>
+    <t>Si actualizan la tabla y cambia mi clase de riesgo, ¿debo cotizar distinto de inmediato?</t>
+  </si>
+  <si>
+    <t>B005</t>
+  </si>
+  <si>
+    <t>Dueño de MiPyme que no entiende el concepto técnico de SST.</t>
+  </si>
+  <si>
+    <t>¿Qué es la Seguridad y Salud en el Trabajo (SST)?</t>
+  </si>
+  <si>
+    <t>B006</t>
+  </si>
+  <si>
+    <t>Empresa que confunde el SG-SST con un simple documento.</t>
+  </si>
+  <si>
+    <t>¿Qué es el Sistema de Gestión de la Seguridad y Salud en el Trabajo (SG-SST)?</t>
+  </si>
+  <si>
+    <t>B007</t>
+  </si>
+  <si>
+    <t>Empresa que ya redactó su política de SST pero no definió objetivos.</t>
+  </si>
+  <si>
+    <t>¿Qué objetivos debe incluir mi política de SST?</t>
+  </si>
+  <si>
+    <t>B008</t>
+  </si>
+  <si>
+    <t>MiPyme que no sabe qué apoyo puede exigirle a su ARL.</t>
+  </si>
+  <si>
+    <t>¿Qué obligaciones tiene mi ARL frente a mi SG-SST?</t>
+  </si>
+  <si>
+    <t>B009</t>
+  </si>
+  <si>
+    <t>Empresa que quiere involucrar a sus trabajadores en el SG-SST.</t>
+  </si>
+  <si>
+    <t>¿Qué responsabilidades tienen mis trabajadores frente al SG-SST?</t>
+  </si>
+  <si>
+    <t>B010</t>
+  </si>
+  <si>
+    <t>Empresa que no sabe cómo archivar los documentos de su SG-SST.</t>
+  </si>
+  <si>
+    <t>¿Cómo debo conservar los documentos y registros del SG-SST?</t>
+  </si>
+  <si>
+    <t>B011</t>
+  </si>
+  <si>
+    <t>Empresa que nunca ha informado a sus trabajadores sobre el SG-SST.</t>
+  </si>
+  <si>
+    <t>¿Qué debo comunicar a mis trabajadores sobre el SG-SST?</t>
+  </si>
+  <si>
+    <t>B012</t>
+  </si>
+  <si>
+    <t>Empresa que va a implementar el SG-SST por primera vez.</t>
+  </si>
+  <si>
+    <t>¿En qué consiste la evaluación inicial del SG-SST?</t>
+  </si>
+  <si>
+    <t>B013</t>
+  </si>
+  <si>
+    <t>Empresa que ya hizo su evaluación inicial y no sabe el siguiente paso.</t>
+  </si>
+  <si>
+    <t>¿Cómo debo planificar mi SG-SST después de la evaluación inicial?</t>
+  </si>
+  <si>
+    <t>B014</t>
+  </si>
+  <si>
+    <t>Empresa que quiere medir el avance de su SG-SST.</t>
+  </si>
+  <si>
+    <t>¿Qué indicadores debo definir para evaluar mi SG-SST?</t>
+  </si>
+  <si>
+    <t>B015</t>
+  </si>
+  <si>
+    <t>Empresa que identificó un riesgo mecánico en un puesto de trabajo.</t>
+  </si>
+  <si>
+    <t>¿Qué tipo de medidas debo priorizar frente a un peligro identificado?</t>
+  </si>
+  <si>
+    <t>B016</t>
+  </si>
+  <si>
+    <t>MiPyme ubicada en una zona con riesgo de sismos o incendios.</t>
+  </si>
+  <si>
+    <t>¿Debo tener un plan de prevención y respuesta ante emergencias?</t>
+  </si>
+  <si>
+    <t>B017</t>
+  </si>
+  <si>
+    <t>Empresa que lleva un año con su SG-SST implementado.</t>
+  </si>
+  <si>
+    <t>¿Debo hacer una auditoría anual de mi SG-SST?</t>
+  </si>
+  <si>
+    <t>B018</t>
+  </si>
+  <si>
+    <t>Dueño de MiPyme que delega todo el SG-SST en un empleado.</t>
+  </si>
+  <si>
+    <t>¿Quién debe revisar el SG-SST y con qué frecuencia?</t>
+  </si>
+  <si>
+    <t>B019</t>
+  </si>
+  <si>
+    <t>Empresa que quiere mejorar continuamente su SG-SST.</t>
+  </si>
+  <si>
+    <t>¿Qué debo hacer para mejorar continuamente mi SG-SST?</t>
+  </si>
+  <si>
+    <t>B020</t>
+  </si>
+  <si>
+    <t>Empresa que acaba de nombrar un responsable de SST.</t>
+  </si>
+  <si>
+    <t>¿Mi responsable de SST debe tomar algún curso obligatorio?</t>
+  </si>
+  <si>
+    <t>B021</t>
+  </si>
+  <si>
+    <t>Empresa de riesgo I que creció de 8 a 15 trabajadores.</t>
+  </si>
+  <si>
+    <t>Si mi empresa crece a 15 trabajadores, ¿qué estándares mínimos debo cumplir ahora?</t>
+  </si>
+  <si>
+    <t>B022</t>
+  </si>
+  <si>
+    <t>Empresa de 20 trabajadores sin persona asignada al SG-SST.</t>
+  </si>
+  <si>
+    <t>¿Quién puede diseñar el SG-SST en una empresa de 20 trabajadores?</t>
+  </si>
+  <si>
+    <t>B023</t>
+  </si>
+  <si>
+    <t>Empresa de 30 trabajadores que busca apoyo externo para su SG-SST.</t>
+  </si>
+  <si>
+    <t>¿Qué apoyo puede recibir mi empresa de 30 trabajadores para el SG-SST?</t>
+  </si>
+  <si>
+    <t>B024</t>
+  </si>
+  <si>
+    <t>Empresa que va a contratar un proveedor externo.</t>
+  </si>
+  <si>
+    <t>¿Puedo exigirle a mi proveedor que cumpla los estándares mínimos de SST?</t>
+  </si>
+  <si>
+    <t>B025</t>
+  </si>
+  <si>
+    <t>Empresa que alcanzó 80 trabajadores.</t>
+  </si>
+  <si>
+    <t>¿Qué estándares mínimos debe cumplir una empresa de más de 50 trabajadores?</t>
+  </si>
+  <si>
+    <t>B026</t>
+  </si>
+  <si>
+    <t>MiPyme que cree que los estándares mínimos son iguales para todas las empresas.</t>
+  </si>
+  <si>
+    <t>¿Los estándares mínimos se ajustan según el tamaño de mi empresa?</t>
+  </si>
+  <si>
+    <t>B027</t>
+  </si>
+  <si>
+    <t>Empresa que ya diseñó su SG-SST con estándares mínimos.</t>
+  </si>
+  <si>
+    <t>¿Qué debe liderar el empleador frente al cumplimiento de los estándares mínimos?</t>
+  </si>
+  <si>
+    <t>B028</t>
+  </si>
+  <si>
+    <t>Empresa con excelente desempeño en SST que quiere destacarse.</t>
+  </si>
+  <si>
+    <t>¿Puede mi empresa obtener un reconocimiento oficial por su desempeño en SST?</t>
+  </si>
+  <si>
+    <t>B029</t>
+  </si>
+  <si>
+    <t>Empresa con trabajadores independientes y en misión además de los de planta.</t>
+  </si>
+  <si>
+    <t>¿Debo contar a los trabajadores independientes y en misión en mis indicadores de SST?</t>
+  </si>
+  <si>
+    <t>B030</t>
+  </si>
+  <si>
+    <t>Empresa que afilia a sus trabajadores a través de una agremiación.</t>
+  </si>
+  <si>
+    <t>¿Es válido afiliar a mis trabajadores a riesgos laborales por medio de una agremiación?</t>
+  </si>
+  <si>
+    <t>B031</t>
+  </si>
+  <si>
+    <t>Empresa que está implementando su SG-SST por fases.</t>
+  </si>
+  <si>
+    <t>¿En qué consisten las fases de adecuación y transición del SG-SST?</t>
+  </si>
+  <si>
+    <t>B032</t>
+  </si>
+  <si>
+    <t>Empresa que se autoevaluó en sus estándares mínimos.</t>
+  </si>
+  <si>
+    <t>¿Cómo se califican los estándares mínimos en la autoevaluación?</t>
+  </si>
+  <si>
+    <t>B033</t>
+  </si>
+  <si>
+    <t>Empresa cuya autoevaluación de estándares mínimos salió con bajo puntaje.</t>
+  </si>
+  <si>
+    <t>Si el resultado de mi autoevaluación no es satisfactorio, ¿qué debo hacer?</t>
+  </si>
+  <si>
+    <t>B034</t>
+  </si>
+  <si>
+    <t>Empresa que quiere saber qué debe medir cada año en SST.</t>
+  </si>
+  <si>
+    <t>¿Qué indicadores mínimos de SST debo registrar cada año?</t>
+  </si>
+  <si>
+    <t>B035</t>
+  </si>
+  <si>
+    <t>Cooperativa de trabajo asociado con un accidente de un trabajador cooperado.</t>
+  </si>
+  <si>
+    <t>¿Esta resolución aplica a las cooperativas de trabajo asociado?</t>
+  </si>
+  <si>
+    <t>B036</t>
+  </si>
+  <si>
+    <t>Una máquina falla pero nadie resulta lesionado ni hay daños.</t>
+  </si>
+  <si>
+    <t>¿Ese hecho se considera un incidente de trabajo?</t>
+  </si>
+  <si>
+    <t>B037</t>
+  </si>
+  <si>
+    <t>Empresa que aún no ha conformado su equipo investigador.</t>
+  </si>
+  <si>
+    <t>¿Qué debo hacer antes de que ocurra un accidente, respecto al equipo investigador?</t>
+  </si>
+  <si>
+    <t>B038</t>
+  </si>
+  <si>
+    <t>Empresa que no tiene un formato definido para investigar accidentes.</t>
+  </si>
+  <si>
+    <t>¿Debo usar un formato específico para investigar los accidentes de trabajo?</t>
+  </si>
+  <si>
+    <t>B039</t>
+  </si>
+  <si>
+    <t>La ARL recomienda medidas correctivas tras un accidente.</t>
+  </si>
+  <si>
+    <t>¿Estoy obligado a implementar las medidas correctivas que recomiende la ARL?</t>
+  </si>
+  <si>
+    <t>B040</t>
+  </si>
+  <si>
+    <t>Empresa pequeña sin metodología propia de investigación de accidentes.</t>
+  </si>
+  <si>
+    <t>¿La ARL debe darme una metodología para investigar accidentes?</t>
+  </si>
+  <si>
+    <t>B041</t>
+  </si>
+  <si>
+    <t>Empresa que quiere adaptar su propia metodología de investigación.</t>
+  </si>
+  <si>
+    <t>¿Puedo usar mi propia metodología para investigar accidentes de trabajo?</t>
+  </si>
+  <si>
+    <t>B042</t>
+  </si>
+  <si>
+    <t>Un trabajador en misión de una empresa temporal sufre un accidente en la empresa usuaria.</t>
+  </si>
+  <si>
+    <t>¿Quién es responsable de investigar ese accidente?</t>
+  </si>
+  <si>
+    <t>B043</t>
+  </si>
+  <si>
+    <t>Empresa terminando el informe de un accidente de trabajo.</t>
+  </si>
+  <si>
+    <t>¿Qué información debe contener el informe de investigación del accidente?</t>
+  </si>
+  <si>
+    <t>B044</t>
+  </si>
+  <si>
+    <t>Investigación de un accidente ya realizada por la empresa.</t>
+  </si>
+  <si>
+    <t>¿Qué debo identificar como causas del accidente en el informe?</t>
+  </si>
+  <si>
+    <t>B045</t>
+  </si>
+  <si>
+    <t>Empresa documentando formalmente su investigación de un accidente.</t>
+  </si>
+  <si>
+    <t>¿Qué datos debe registrar el informe sobre la investigación misma (lugar, fecha, investigadores)?</t>
+  </si>
+  <si>
+    <t>B046</t>
+  </si>
+  <si>
+    <t>Empresa que no investigó un accidente grave ocurrido en sus instalaciones.</t>
+  </si>
+  <si>
+    <t>¿Qué consecuencia tiene no cumplir con esta resolución?</t>
+  </si>
+  <si>
+    <t>B047</t>
+  </si>
+  <si>
+    <t>Trabajador víctima de comentarios ofensivos reiterados por parte de un compañero.</t>
+  </si>
+  <si>
+    <t>¿Qué busca proteger la Ley 1010 de 2006?</t>
+  </si>
+  <si>
+    <t>B048</t>
+  </si>
+  <si>
+    <t>Un jefe que acosó pero corrigió su conducta y se disculpó.</t>
+  </si>
+  <si>
+    <t>¿Existen atenuantes si el acoso laboral ya está probado?</t>
+  </si>
+  <si>
+    <t>B049</t>
+  </si>
+  <si>
+    <t>Un directivo de alto cargo que acosa a un subordinado.</t>
+  </si>
+  <si>
+    <t>¿Se agrava la sanción si el acosador tiene un cargo jerárquico alto?</t>
+  </si>
+  <si>
+    <t>B050</t>
+  </si>
+  <si>
+    <t>Un compañero de trabajo, sin ser jefe, acosa a otro trabajador.</t>
+  </si>
+  <si>
+    <t>¿Puede un compañero de trabajo ser sujeto activo de acoso laboral?</t>
+  </si>
+  <si>
+    <t>B051</t>
+  </si>
+  <si>
+    <t>Un jefe le asigna cargas de trabajo excesivas de forma reiterada buscando que renuncie.</t>
+  </si>
+  <si>
+    <t>¿Esa conducta corresponde a una modalidad específica de acoso laboral?</t>
+  </si>
+  <si>
+    <t>B052</t>
+  </si>
+  <si>
+    <t>Un compañero oculta documentos necesarios para que otro no pueda cumplir su labor.</t>
+  </si>
+  <si>
+    <t>¿Esa conducta constituye una modalidad de acoso laboral?</t>
+  </si>
+  <si>
+    <t>B053</t>
+  </si>
+  <si>
+    <t>Un trabajador que denunció acoso laboral teme represalias de su jefe.</t>
+  </si>
+  <si>
+    <t>¿Qué garantías tengo si denuncio acoso laboral?</t>
+  </si>
+  <si>
+    <t>B054</t>
+  </si>
+  <si>
+    <t>Se va a sancionar un caso de acoso laboral ya acreditado.</t>
+  </si>
+  <si>
+    <t>¿Qué procedimiento se sigue para sancionar el acoso laboral?</t>
+  </si>
+  <si>
+    <t>B055</t>
+  </si>
+  <si>
+    <t>Un trabajador presenta una queja de acoso laboral sin fundamento real.</t>
+  </si>
+  <si>
+    <t>¿Qué pasa si mi queja de acoso laboral resulta infundada?</t>
+  </si>
+  <si>
+    <t>B056</t>
+  </si>
+  <si>
+    <t>Un trabajador quiere denunciar un acoso ocurrido hace dos años.</t>
+  </si>
+  <si>
+    <t>¿Cuánto tiempo tengo para denunciar el acoso laboral?</t>
+  </si>
+  <si>
+    <t>B057</t>
+  </si>
+  <si>
+    <t>Empresa con trabajadores vinculados por contrato de prestación de servicios.</t>
+  </si>
+  <si>
+    <t>¿Quiénes están obligados a afiliarse al Sistema General de Riesgos Laborales?</t>
+  </si>
+  <si>
+    <t>B058</t>
+  </si>
+  <si>
+    <t>Trabajador diagnosticado con una enfermedad laboral.</t>
+  </si>
+  <si>
+    <t>¿Cómo se calcula el ingreso base para pagarle por una enfermedad laboral?</t>
+  </si>
+  <si>
+    <t>B059</t>
+  </si>
+  <si>
+    <t>Trabajador incapacitado mientras se decide si el origen es laboral o común.</t>
+  </si>
+  <si>
+    <t>¿Quién me paga la incapacidad mientras se define el origen laboral o común?</t>
+  </si>
+  <si>
+    <t>B060</t>
+  </si>
+  <si>
+    <t>Empresa que contrata a un trabajador independiente por prestación de servicios.</t>
+  </si>
+  <si>
+    <t>¿También debo cotizar riesgos laborales por un contratista independiente?</t>
+  </si>
+  <si>
+    <t>B061</t>
+  </si>
+  <si>
+    <t>Empresa que se atrasó en el pago de aportes a su ARL.</t>
+  </si>
+  <si>
+    <t>Si me atraso en el pago de aportes, ¿pierdo automáticamente la afiliación de mis trabajadores?</t>
+  </si>
+  <si>
+    <t>B062</t>
+  </si>
+  <si>
+    <t>La ARL debe reportar sus resultados de prevención al Ministerio del Trabajo.</t>
+  </si>
+  <si>
+    <t>¿Qué debe reportar mi ARL sobre sus actividades de promoción y prevención?</t>
+  </si>
+  <si>
+    <t>B063</t>
+  </si>
+  <si>
+    <t>Empresa que quiere saber qué debe darle su ARL en materia de prevención.</t>
+  </si>
+  <si>
+    <t>¿Qué servicios mínimos de promoción y prevención debe prestarme mi ARL?</t>
+  </si>
+  <si>
+    <t>B064</t>
+  </si>
+  <si>
+    <t>Empresa que incumple normas del Sistema de Riesgos Laborales.</t>
+  </si>
+  <si>
+    <t>¿Qué sanciones prevé la ley por incumplir el Sistema de Riesgos Laborales?</t>
+  </si>
+  <si>
+    <t>B065</t>
+  </si>
+  <si>
+    <t>Autoridad que realiza visitas de verificación de estándares en la empresa.</t>
+  </si>
+  <si>
+    <t>¿Pueden hacerme visitas de verificación del cumplimiento en riesgos laborales?</t>
+  </si>
+  <si>
+    <t>B066</t>
+  </si>
+  <si>
+    <t>Empresa clasificada de alto riesgo que se pregunta si recibe trato distinto a una de riesgo I.</t>
+  </si>
+  <si>
+    <t>¿Reciben las empresas de alto riesgo una supervisión distinta a las de riesgo I?</t>
+  </si>
+  <si>
+    <t>B067</t>
+  </si>
+  <si>
+    <t>Empresa con dos sucursales que quiere organizar comités separados.</t>
+  </si>
+  <si>
+    <t>¿Puedo conformar un Comité distinto para cada sede de mi empresa?</t>
+  </si>
+  <si>
+    <t>B068</t>
+  </si>
+  <si>
+    <t>Empresa que va a conformar su primer Comité Paritario.</t>
+  </si>
+  <si>
+    <t>¿Cómo se eligen los representantes del Comité?</t>
+  </si>
+  <si>
+    <t>B069</t>
+  </si>
+  <si>
+    <t>Reunión del Comité con solo la mitad de sus miembros presentes.</t>
+  </si>
+  <si>
+    <t>¿Con cuántos miembros puede sesionar válidamente el Comité?</t>
+  </si>
+  <si>
+    <t>B070</t>
+  </si>
+  <si>
+    <t>Comité recién conformado que aún no ha nombrado presidente.</t>
+  </si>
+  <si>
+    <t>¿Quién designa al Presidente del Comité?</t>
+  </si>
+  <si>
+    <t>B071</t>
+  </si>
+  <si>
+    <t>Un trabajador quiere llevar una queja disciplinaria al Comité.</t>
+  </si>
+  <si>
+    <t>¿El Comité puede resolver asuntos disciplinarios o contractuales de los trabajadores?</t>
+  </si>
+  <si>
+    <t>B072</t>
+  </si>
+  <si>
+    <t>Comité ya conformado que quiere conocer el alcance de sus funciones.</t>
+  </si>
+  <si>
+    <t>¿Cuáles son las funciones del Comité?</t>
+  </si>
+  <si>
+    <t>B073</t>
+  </si>
+  <si>
+    <t>Empresa que ya tiene su Comité conformado.</t>
+  </si>
+  <si>
+    <t>¿Qué obligaciones tiene el empleador frente al Comité?</t>
+  </si>
+  <si>
+    <t>B074</t>
+  </si>
+  <si>
+    <t>Trabajadores que son miembros del Comité.</t>
+  </si>
+  <si>
+    <t>¿Qué obligaciones tienen los trabajadores frente al Comité?</t>
+  </si>
+  <si>
+    <t>B075</t>
+  </si>
+  <si>
+    <t>Empresa que no sabe cuántos tipos de evaluación médica ocupacional existen.</t>
+  </si>
+  <si>
+    <t>¿Qué tipos de evaluaciones médicas ocupacionales debo realizar?</t>
+  </si>
+  <si>
+    <t>B076</t>
+  </si>
+  <si>
+    <t>Trabajador que lleva tres años en el mismo puesto sin cambiar de cargo.</t>
+  </si>
+  <si>
+    <t>¿Debo hacerle exámenes médicos periódicos aunque no cambie de cargo?</t>
+  </si>
+  <si>
+    <t>B077</t>
+  </si>
+  <si>
+    <t>Empresa que va a contratar el servicio de evaluaciones médicas ocupacionales.</t>
+  </si>
+  <si>
+    <t>¿Quién puede realizar las evaluaciones médicas ocupacionales de mis trabajadores?</t>
+  </si>
+  <si>
+    <t>B078</t>
+  </si>
+  <si>
+    <t>Trabajador expuesto a ruido o sustancias químicas en su labor.</t>
+  </si>
+  <si>
+    <t>¿Debo hacerle exámenes médicos específicos según el riesgo al que está expuesto?</t>
+  </si>
+  <si>
+    <t>B079</t>
+  </si>
+  <si>
+    <t>Trabajador con varios exámenes ocupacionales realizados durante su vida laboral.</t>
+  </si>
+  <si>
+    <t>¿Qué es la historia clínica ocupacional?</t>
+  </si>
+  <si>
+    <t>B080</t>
+  </si>
+  <si>
+    <t>El empleador quiere revisar la historia clínica de un trabajador.</t>
+  </si>
+  <si>
+    <t>¿Puedo como empleador acceder a la historia clínica ocupacional de mis trabajadores?</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1274,6 +1995,12 @@
       <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="DilleniaUPC"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
       <charset val="1"/>
     </font>
   </fonts>
@@ -1432,7 +2159,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1506,6 +2233,10 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -3533,9 +4264,1392 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF072275-00C3-4942-9129-BD41CE62AD44}">
-  <dimension ref="A1"/>
+  <dimension ref="B5:F85"/>
   <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col min="3" max="3" width="23.42578125" customWidth="1"/>
+    <col min="4" max="6" width="36.5703125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="5" spans="2:6" ht="18">
+      <c r="B5" s="14" t="s">
+        <v>30</v>
+      </c>
+      <c r="C5" s="14" t="s">
+        <v>31</v>
+      </c>
+      <c r="D5" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="E5" s="14" t="s">
+        <v>34</v>
+      </c>
+      <c r="F5" s="14" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="6" spans="2:6" ht="27">
+      <c r="B6" s="31" t="s">
+        <v>351</v>
+      </c>
+      <c r="C6" s="31" t="s">
+        <v>6</v>
+      </c>
+      <c r="D6" s="32" t="s">
+        <v>352</v>
+      </c>
+      <c r="E6" s="32" t="s">
+        <v>353</v>
+      </c>
+      <c r="F6" s="32" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="2:6" ht="27">
+      <c r="B7" s="31" t="s">
+        <v>354</v>
+      </c>
+      <c r="C7" s="31" t="s">
+        <v>6</v>
+      </c>
+      <c r="D7" s="32" t="s">
+        <v>355</v>
+      </c>
+      <c r="E7" s="32" t="s">
+        <v>356</v>
+      </c>
+      <c r="F7" s="32" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="2:6" ht="27">
+      <c r="B8" s="31" t="s">
+        <v>357</v>
+      </c>
+      <c r="C8" s="31" t="s">
+        <v>6</v>
+      </c>
+      <c r="D8" s="32" t="s">
+        <v>358</v>
+      </c>
+      <c r="E8" s="32" t="s">
+        <v>359</v>
+      </c>
+      <c r="F8" s="32" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="2:6" ht="27">
+      <c r="B9" s="31" t="s">
+        <v>360</v>
+      </c>
+      <c r="C9" s="31" t="s">
+        <v>6</v>
+      </c>
+      <c r="D9" s="32" t="s">
+        <v>361</v>
+      </c>
+      <c r="E9" s="32" t="s">
+        <v>362</v>
+      </c>
+      <c r="F9" s="32" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10" spans="2:6" ht="27">
+      <c r="B10" s="31" t="s">
+        <v>363</v>
+      </c>
+      <c r="C10" s="31" t="s">
+        <v>10</v>
+      </c>
+      <c r="D10" s="32" t="s">
+        <v>364</v>
+      </c>
+      <c r="E10" s="32" t="s">
+        <v>365</v>
+      </c>
+      <c r="F10" s="32" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="2:6" ht="27">
+      <c r="B11" s="31" t="s">
+        <v>366</v>
+      </c>
+      <c r="C11" s="31" t="s">
+        <v>10</v>
+      </c>
+      <c r="D11" s="32" t="s">
+        <v>367</v>
+      </c>
+      <c r="E11" s="32" t="s">
+        <v>368</v>
+      </c>
+      <c r="F11" s="32" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="2:6" ht="27">
+      <c r="B12" s="31" t="s">
+        <v>369</v>
+      </c>
+      <c r="C12" s="31" t="s">
+        <v>10</v>
+      </c>
+      <c r="D12" s="32" t="s">
+        <v>370</v>
+      </c>
+      <c r="E12" s="32" t="s">
+        <v>371</v>
+      </c>
+      <c r="F12" s="32" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="2:6" ht="27">
+      <c r="B13" s="31" t="s">
+        <v>372</v>
+      </c>
+      <c r="C13" s="31" t="s">
+        <v>10</v>
+      </c>
+      <c r="D13" s="32" t="s">
+        <v>373</v>
+      </c>
+      <c r="E13" s="32" t="s">
+        <v>374</v>
+      </c>
+      <c r="F13" s="32" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14" spans="2:6" ht="27">
+      <c r="B14" s="31" t="s">
+        <v>375</v>
+      </c>
+      <c r="C14" s="31" t="s">
+        <v>10</v>
+      </c>
+      <c r="D14" s="32" t="s">
+        <v>376</v>
+      </c>
+      <c r="E14" s="32" t="s">
+        <v>377</v>
+      </c>
+      <c r="F14" s="32" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15" spans="2:6" ht="27">
+      <c r="B15" s="31" t="s">
+        <v>378</v>
+      </c>
+      <c r="C15" s="31" t="s">
+        <v>10</v>
+      </c>
+      <c r="D15" s="32" t="s">
+        <v>379</v>
+      </c>
+      <c r="E15" s="32" t="s">
+        <v>380</v>
+      </c>
+      <c r="F15" s="32" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="16" spans="2:6" ht="27">
+      <c r="B16" s="31" t="s">
+        <v>381</v>
+      </c>
+      <c r="C16" s="31" t="s">
+        <v>10</v>
+      </c>
+      <c r="D16" s="32" t="s">
+        <v>382</v>
+      </c>
+      <c r="E16" s="32" t="s">
+        <v>383</v>
+      </c>
+      <c r="F16" s="32" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="17" spans="2:6" ht="27">
+      <c r="B17" s="31" t="s">
+        <v>384</v>
+      </c>
+      <c r="C17" s="31" t="s">
+        <v>10</v>
+      </c>
+      <c r="D17" s="32" t="s">
+        <v>385</v>
+      </c>
+      <c r="E17" s="32" t="s">
+        <v>386</v>
+      </c>
+      <c r="F17" s="32" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="18" spans="2:6" ht="27">
+      <c r="B18" s="31" t="s">
+        <v>387</v>
+      </c>
+      <c r="C18" s="31" t="s">
+        <v>10</v>
+      </c>
+      <c r="D18" s="32" t="s">
+        <v>388</v>
+      </c>
+      <c r="E18" s="32" t="s">
+        <v>389</v>
+      </c>
+      <c r="F18" s="32" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="19" spans="2:6" ht="27">
+      <c r="B19" s="31" t="s">
+        <v>390</v>
+      </c>
+      <c r="C19" s="31" t="s">
+        <v>10</v>
+      </c>
+      <c r="D19" s="32" t="s">
+        <v>391</v>
+      </c>
+      <c r="E19" s="32" t="s">
+        <v>392</v>
+      </c>
+      <c r="F19" s="32" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="20" spans="2:6" ht="27">
+      <c r="B20" s="31" t="s">
+        <v>393</v>
+      </c>
+      <c r="C20" s="31" t="s">
+        <v>10</v>
+      </c>
+      <c r="D20" s="32" t="s">
+        <v>394</v>
+      </c>
+      <c r="E20" s="32" t="s">
+        <v>395</v>
+      </c>
+      <c r="F20" s="32" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="21" spans="2:6" ht="27">
+      <c r="B21" s="31" t="s">
+        <v>396</v>
+      </c>
+      <c r="C21" s="31" t="s">
+        <v>10</v>
+      </c>
+      <c r="D21" s="32" t="s">
+        <v>397</v>
+      </c>
+      <c r="E21" s="32" t="s">
+        <v>398</v>
+      </c>
+      <c r="F21" s="32" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="22" spans="2:6" ht="27">
+      <c r="B22" s="31" t="s">
+        <v>399</v>
+      </c>
+      <c r="C22" s="31" t="s">
+        <v>10</v>
+      </c>
+      <c r="D22" s="32" t="s">
+        <v>400</v>
+      </c>
+      <c r="E22" s="32" t="s">
+        <v>401</v>
+      </c>
+      <c r="F22" s="32" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="23" spans="2:6" ht="27">
+      <c r="B23" s="31" t="s">
+        <v>402</v>
+      </c>
+      <c r="C23" s="31" t="s">
+        <v>10</v>
+      </c>
+      <c r="D23" s="32" t="s">
+        <v>403</v>
+      </c>
+      <c r="E23" s="32" t="s">
+        <v>404</v>
+      </c>
+      <c r="F23" s="32" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="24" spans="2:6" ht="27">
+      <c r="B24" s="31" t="s">
+        <v>405</v>
+      </c>
+      <c r="C24" s="31" t="s">
+        <v>10</v>
+      </c>
+      <c r="D24" s="32" t="s">
+        <v>406</v>
+      </c>
+      <c r="E24" s="32" t="s">
+        <v>407</v>
+      </c>
+      <c r="F24" s="32" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="25" spans="2:6" ht="27">
+      <c r="B25" s="31" t="s">
+        <v>408</v>
+      </c>
+      <c r="C25" s="31" t="s">
+        <v>10</v>
+      </c>
+      <c r="D25" s="32" t="s">
+        <v>409</v>
+      </c>
+      <c r="E25" s="32" t="s">
+        <v>410</v>
+      </c>
+      <c r="F25" s="32" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="26" spans="2:6" ht="27">
+      <c r="B26" s="31" t="s">
+        <v>411</v>
+      </c>
+      <c r="C26" s="31" t="s">
+        <v>19</v>
+      </c>
+      <c r="D26" s="32" t="s">
+        <v>412</v>
+      </c>
+      <c r="E26" s="32" t="s">
+        <v>413</v>
+      </c>
+      <c r="F26" s="32" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="27" spans="2:6" ht="27">
+      <c r="B27" s="31" t="s">
+        <v>414</v>
+      </c>
+      <c r="C27" s="31" t="s">
+        <v>19</v>
+      </c>
+      <c r="D27" s="32" t="s">
+        <v>415</v>
+      </c>
+      <c r="E27" s="32" t="s">
+        <v>416</v>
+      </c>
+      <c r="F27" s="32" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="28" spans="2:6" ht="27">
+      <c r="B28" s="31" t="s">
+        <v>417</v>
+      </c>
+      <c r="C28" s="31" t="s">
+        <v>19</v>
+      </c>
+      <c r="D28" s="32" t="s">
+        <v>418</v>
+      </c>
+      <c r="E28" s="32" t="s">
+        <v>419</v>
+      </c>
+      <c r="F28" s="32" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="29" spans="2:6" ht="27">
+      <c r="B29" s="31" t="s">
+        <v>420</v>
+      </c>
+      <c r="C29" s="31" t="s">
+        <v>19</v>
+      </c>
+      <c r="D29" s="32" t="s">
+        <v>421</v>
+      </c>
+      <c r="E29" s="32" t="s">
+        <v>422</v>
+      </c>
+      <c r="F29" s="32" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="30" spans="2:6" ht="27">
+      <c r="B30" s="31" t="s">
+        <v>423</v>
+      </c>
+      <c r="C30" s="31" t="s">
+        <v>19</v>
+      </c>
+      <c r="D30" s="32" t="s">
+        <v>424</v>
+      </c>
+      <c r="E30" s="32" t="s">
+        <v>425</v>
+      </c>
+      <c r="F30" s="32" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="31" spans="2:6" ht="27">
+      <c r="B31" s="31" t="s">
+        <v>426</v>
+      </c>
+      <c r="C31" s="31" t="s">
+        <v>19</v>
+      </c>
+      <c r="D31" s="32" t="s">
+        <v>427</v>
+      </c>
+      <c r="E31" s="32" t="s">
+        <v>428</v>
+      </c>
+      <c r="F31" s="32" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="32" spans="2:6" ht="27">
+      <c r="B32" s="31" t="s">
+        <v>429</v>
+      </c>
+      <c r="C32" s="31" t="s">
+        <v>19</v>
+      </c>
+      <c r="D32" s="32" t="s">
+        <v>430</v>
+      </c>
+      <c r="E32" s="32" t="s">
+        <v>431</v>
+      </c>
+      <c r="F32" s="32" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="33" spans="2:6" ht="40.5">
+      <c r="B33" s="31" t="s">
+        <v>432</v>
+      </c>
+      <c r="C33" s="31" t="s">
+        <v>19</v>
+      </c>
+      <c r="D33" s="32" t="s">
+        <v>433</v>
+      </c>
+      <c r="E33" s="32" t="s">
+        <v>434</v>
+      </c>
+      <c r="F33" s="32" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="34" spans="2:6" ht="40.5">
+      <c r="B34" s="31" t="s">
+        <v>435</v>
+      </c>
+      <c r="C34" s="31" t="s">
+        <v>19</v>
+      </c>
+      <c r="D34" s="32" t="s">
+        <v>436</v>
+      </c>
+      <c r="E34" s="32" t="s">
+        <v>437</v>
+      </c>
+      <c r="F34" s="32" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="35" spans="2:6" ht="27">
+      <c r="B35" s="31" t="s">
+        <v>438</v>
+      </c>
+      <c r="C35" s="31" t="s">
+        <v>19</v>
+      </c>
+      <c r="D35" s="32" t="s">
+        <v>439</v>
+      </c>
+      <c r="E35" s="32" t="s">
+        <v>440</v>
+      </c>
+      <c r="F35" s="32" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="36" spans="2:6" ht="27">
+      <c r="B36" s="31" t="s">
+        <v>441</v>
+      </c>
+      <c r="C36" s="31" t="s">
+        <v>19</v>
+      </c>
+      <c r="D36" s="32" t="s">
+        <v>442</v>
+      </c>
+      <c r="E36" s="32" t="s">
+        <v>443</v>
+      </c>
+      <c r="F36" s="32" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="37" spans="2:6" ht="27">
+      <c r="B37" s="31" t="s">
+        <v>444</v>
+      </c>
+      <c r="C37" s="31" t="s">
+        <v>19</v>
+      </c>
+      <c r="D37" s="32" t="s">
+        <v>445</v>
+      </c>
+      <c r="E37" s="32" t="s">
+        <v>446</v>
+      </c>
+      <c r="F37" s="32" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="38" spans="2:6" ht="27">
+      <c r="B38" s="31" t="s">
+        <v>447</v>
+      </c>
+      <c r="C38" s="31" t="s">
+        <v>19</v>
+      </c>
+      <c r="D38" s="32" t="s">
+        <v>448</v>
+      </c>
+      <c r="E38" s="32" t="s">
+        <v>449</v>
+      </c>
+      <c r="F38" s="32" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="39" spans="2:6" ht="27">
+      <c r="B39" s="31" t="s">
+        <v>450</v>
+      </c>
+      <c r="C39" s="31" t="s">
+        <v>19</v>
+      </c>
+      <c r="D39" s="32" t="s">
+        <v>451</v>
+      </c>
+      <c r="E39" s="32" t="s">
+        <v>452</v>
+      </c>
+      <c r="F39" s="32" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="40" spans="2:6" ht="27">
+      <c r="B40" s="31" t="s">
+        <v>453</v>
+      </c>
+      <c r="C40" s="31" t="s">
+        <v>22</v>
+      </c>
+      <c r="D40" s="32" t="s">
+        <v>454</v>
+      </c>
+      <c r="E40" s="32" t="s">
+        <v>455</v>
+      </c>
+      <c r="F40" s="32" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="41" spans="2:6" ht="27">
+      <c r="B41" s="31" t="s">
+        <v>456</v>
+      </c>
+      <c r="C41" s="31" t="s">
+        <v>22</v>
+      </c>
+      <c r="D41" s="32" t="s">
+        <v>457</v>
+      </c>
+      <c r="E41" s="32" t="s">
+        <v>458</v>
+      </c>
+      <c r="F41" s="32" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="42" spans="2:6" ht="27">
+      <c r="B42" s="31" t="s">
+        <v>459</v>
+      </c>
+      <c r="C42" s="31" t="s">
+        <v>22</v>
+      </c>
+      <c r="D42" s="32" t="s">
+        <v>460</v>
+      </c>
+      <c r="E42" s="32" t="s">
+        <v>461</v>
+      </c>
+      <c r="F42" s="32" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="43" spans="2:6" ht="27">
+      <c r="B43" s="31" t="s">
+        <v>462</v>
+      </c>
+      <c r="C43" s="31" t="s">
+        <v>22</v>
+      </c>
+      <c r="D43" s="32" t="s">
+        <v>463</v>
+      </c>
+      <c r="E43" s="32" t="s">
+        <v>464</v>
+      </c>
+      <c r="F43" s="32" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="44" spans="2:6" ht="27">
+      <c r="B44" s="31" t="s">
+        <v>465</v>
+      </c>
+      <c r="C44" s="31" t="s">
+        <v>22</v>
+      </c>
+      <c r="D44" s="32" t="s">
+        <v>466</v>
+      </c>
+      <c r="E44" s="32" t="s">
+        <v>467</v>
+      </c>
+      <c r="F44" s="32" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="45" spans="2:6" ht="27">
+      <c r="B45" s="31" t="s">
+        <v>468</v>
+      </c>
+      <c r="C45" s="31" t="s">
+        <v>22</v>
+      </c>
+      <c r="D45" s="32" t="s">
+        <v>469</v>
+      </c>
+      <c r="E45" s="32" t="s">
+        <v>470</v>
+      </c>
+      <c r="F45" s="32" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="46" spans="2:6" ht="27">
+      <c r="B46" s="31" t="s">
+        <v>471</v>
+      </c>
+      <c r="C46" s="31" t="s">
+        <v>22</v>
+      </c>
+      <c r="D46" s="32" t="s">
+        <v>472</v>
+      </c>
+      <c r="E46" s="32" t="s">
+        <v>473</v>
+      </c>
+      <c r="F46" s="32" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="47" spans="2:6" ht="40.5">
+      <c r="B47" s="31" t="s">
+        <v>474</v>
+      </c>
+      <c r="C47" s="31" t="s">
+        <v>22</v>
+      </c>
+      <c r="D47" s="32" t="s">
+        <v>475</v>
+      </c>
+      <c r="E47" s="32" t="s">
+        <v>476</v>
+      </c>
+      <c r="F47" s="32" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="48" spans="2:6" ht="27">
+      <c r="B48" s="31" t="s">
+        <v>477</v>
+      </c>
+      <c r="C48" s="31" t="s">
+        <v>22</v>
+      </c>
+      <c r="D48" s="32" t="s">
+        <v>478</v>
+      </c>
+      <c r="E48" s="32" t="s">
+        <v>479</v>
+      </c>
+      <c r="F48" s="32" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="49" spans="2:6" ht="27">
+      <c r="B49" s="31" t="s">
+        <v>480</v>
+      </c>
+      <c r="C49" s="31" t="s">
+        <v>22</v>
+      </c>
+      <c r="D49" s="32" t="s">
+        <v>481</v>
+      </c>
+      <c r="E49" s="32" t="s">
+        <v>482</v>
+      </c>
+      <c r="F49" s="32" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="50" spans="2:6" ht="40.5">
+      <c r="B50" s="31" t="s">
+        <v>483</v>
+      </c>
+      <c r="C50" s="31" t="s">
+        <v>22</v>
+      </c>
+      <c r="D50" s="32" t="s">
+        <v>484</v>
+      </c>
+      <c r="E50" s="32" t="s">
+        <v>485</v>
+      </c>
+      <c r="F50" s="32" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="51" spans="2:6" ht="27">
+      <c r="B51" s="31" t="s">
+        <v>486</v>
+      </c>
+      <c r="C51" s="31" t="s">
+        <v>22</v>
+      </c>
+      <c r="D51" s="32" t="s">
+        <v>487</v>
+      </c>
+      <c r="E51" s="32" t="s">
+        <v>488</v>
+      </c>
+      <c r="F51" s="32" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="52" spans="2:6" ht="27">
+      <c r="B52" s="31" t="s">
+        <v>489</v>
+      </c>
+      <c r="C52" s="31" t="s">
+        <v>13</v>
+      </c>
+      <c r="D52" s="32" t="s">
+        <v>490</v>
+      </c>
+      <c r="E52" s="32" t="s">
+        <v>491</v>
+      </c>
+      <c r="F52" s="32" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="53" spans="2:6" ht="27">
+      <c r="B53" s="31" t="s">
+        <v>492</v>
+      </c>
+      <c r="C53" s="31" t="s">
+        <v>13</v>
+      </c>
+      <c r="D53" s="32" t="s">
+        <v>493</v>
+      </c>
+      <c r="E53" s="32" t="s">
+        <v>494</v>
+      </c>
+      <c r="F53" s="32" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="54" spans="2:6" ht="27">
+      <c r="B54" s="31" t="s">
+        <v>495</v>
+      </c>
+      <c r="C54" s="31" t="s">
+        <v>13</v>
+      </c>
+      <c r="D54" s="32" t="s">
+        <v>496</v>
+      </c>
+      <c r="E54" s="32" t="s">
+        <v>497</v>
+      </c>
+      <c r="F54" s="32" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="55" spans="2:6" ht="27">
+      <c r="B55" s="31" t="s">
+        <v>498</v>
+      </c>
+      <c r="C55" s="31" t="s">
+        <v>13</v>
+      </c>
+      <c r="D55" s="32" t="s">
+        <v>499</v>
+      </c>
+      <c r="E55" s="32" t="s">
+        <v>500</v>
+      </c>
+      <c r="F55" s="32" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="56" spans="2:6" ht="27">
+      <c r="B56" s="31" t="s">
+        <v>501</v>
+      </c>
+      <c r="C56" s="31" t="s">
+        <v>13</v>
+      </c>
+      <c r="D56" s="32" t="s">
+        <v>502</v>
+      </c>
+      <c r="E56" s="32" t="s">
+        <v>503</v>
+      </c>
+      <c r="F56" s="32" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="57" spans="2:6" ht="27">
+      <c r="B57" s="31" t="s">
+        <v>504</v>
+      </c>
+      <c r="C57" s="31" t="s">
+        <v>13</v>
+      </c>
+      <c r="D57" s="32" t="s">
+        <v>505</v>
+      </c>
+      <c r="E57" s="32" t="s">
+        <v>506</v>
+      </c>
+      <c r="F57" s="32" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="58" spans="2:6" ht="27">
+      <c r="B58" s="31" t="s">
+        <v>507</v>
+      </c>
+      <c r="C58" s="31" t="s">
+        <v>13</v>
+      </c>
+      <c r="D58" s="32" t="s">
+        <v>508</v>
+      </c>
+      <c r="E58" s="32" t="s">
+        <v>509</v>
+      </c>
+      <c r="F58" s="32" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="59" spans="2:6" ht="27">
+      <c r="B59" s="31" t="s">
+        <v>510</v>
+      </c>
+      <c r="C59" s="31" t="s">
+        <v>13</v>
+      </c>
+      <c r="D59" s="32" t="s">
+        <v>511</v>
+      </c>
+      <c r="E59" s="32" t="s">
+        <v>512</v>
+      </c>
+      <c r="F59" s="32" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="60" spans="2:6" ht="27">
+      <c r="B60" s="31" t="s">
+        <v>513</v>
+      </c>
+      <c r="C60" s="31" t="s">
+        <v>13</v>
+      </c>
+      <c r="D60" s="32" t="s">
+        <v>514</v>
+      </c>
+      <c r="E60" s="32" t="s">
+        <v>515</v>
+      </c>
+      <c r="F60" s="32" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="61" spans="2:6" ht="27">
+      <c r="B61" s="31" t="s">
+        <v>516</v>
+      </c>
+      <c r="C61" s="31" t="s">
+        <v>13</v>
+      </c>
+      <c r="D61" s="32" t="s">
+        <v>517</v>
+      </c>
+      <c r="E61" s="32" t="s">
+        <v>518</v>
+      </c>
+      <c r="F61" s="32" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="62" spans="2:6" ht="27">
+      <c r="B62" s="31" t="s">
+        <v>519</v>
+      </c>
+      <c r="C62" s="31" t="s">
+        <v>16</v>
+      </c>
+      <c r="D62" s="32" t="s">
+        <v>520</v>
+      </c>
+      <c r="E62" s="32" t="s">
+        <v>521</v>
+      </c>
+      <c r="F62" s="32" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="63" spans="2:6" ht="27">
+      <c r="B63" s="31" t="s">
+        <v>522</v>
+      </c>
+      <c r="C63" s="31" t="s">
+        <v>16</v>
+      </c>
+      <c r="D63" s="32" t="s">
+        <v>523</v>
+      </c>
+      <c r="E63" s="32" t="s">
+        <v>524</v>
+      </c>
+      <c r="F63" s="32" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="64" spans="2:6" ht="27">
+      <c r="B64" s="31" t="s">
+        <v>525</v>
+      </c>
+      <c r="C64" s="31" t="s">
+        <v>16</v>
+      </c>
+      <c r="D64" s="32" t="s">
+        <v>526</v>
+      </c>
+      <c r="E64" s="32" t="s">
+        <v>527</v>
+      </c>
+      <c r="F64" s="32" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="65" spans="2:6" ht="27">
+      <c r="B65" s="31" t="s">
+        <v>528</v>
+      </c>
+      <c r="C65" s="31" t="s">
+        <v>16</v>
+      </c>
+      <c r="D65" s="32" t="s">
+        <v>529</v>
+      </c>
+      <c r="E65" s="32" t="s">
+        <v>530</v>
+      </c>
+      <c r="F65" s="32" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="66" spans="2:6" ht="40.5">
+      <c r="B66" s="31" t="s">
+        <v>531</v>
+      </c>
+      <c r="C66" s="31" t="s">
+        <v>16</v>
+      </c>
+      <c r="D66" s="32" t="s">
+        <v>532</v>
+      </c>
+      <c r="E66" s="32" t="s">
+        <v>533</v>
+      </c>
+      <c r="F66" s="32" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="67" spans="2:6" ht="27">
+      <c r="B67" s="31" t="s">
+        <v>534</v>
+      </c>
+      <c r="C67" s="31" t="s">
+        <v>16</v>
+      </c>
+      <c r="D67" s="32" t="s">
+        <v>535</v>
+      </c>
+      <c r="E67" s="32" t="s">
+        <v>536</v>
+      </c>
+      <c r="F67" s="32" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="68" spans="2:6" ht="27">
+      <c r="B68" s="31" t="s">
+        <v>537</v>
+      </c>
+      <c r="C68" s="31" t="s">
+        <v>16</v>
+      </c>
+      <c r="D68" s="32" t="s">
+        <v>538</v>
+      </c>
+      <c r="E68" s="32" t="s">
+        <v>539</v>
+      </c>
+      <c r="F68" s="32" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="69" spans="2:6" ht="27">
+      <c r="B69" s="31" t="s">
+        <v>540</v>
+      </c>
+      <c r="C69" s="31" t="s">
+        <v>16</v>
+      </c>
+      <c r="D69" s="32" t="s">
+        <v>541</v>
+      </c>
+      <c r="E69" s="32" t="s">
+        <v>542</v>
+      </c>
+      <c r="F69" s="32" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="70" spans="2:6" ht="27">
+      <c r="B70" s="31" t="s">
+        <v>543</v>
+      </c>
+      <c r="C70" s="31" t="s">
+        <v>16</v>
+      </c>
+      <c r="D70" s="32" t="s">
+        <v>544</v>
+      </c>
+      <c r="E70" s="32" t="s">
+        <v>545</v>
+      </c>
+      <c r="F70" s="32" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="71" spans="2:6" ht="40.5">
+      <c r="B71" s="31" t="s">
+        <v>546</v>
+      </c>
+      <c r="C71" s="31" t="s">
+        <v>16</v>
+      </c>
+      <c r="D71" s="32" t="s">
+        <v>547</v>
+      </c>
+      <c r="E71" s="32" t="s">
+        <v>548</v>
+      </c>
+      <c r="F71" s="32" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="72" spans="2:6" ht="27">
+      <c r="B72" s="31" t="s">
+        <v>549</v>
+      </c>
+      <c r="C72" s="31" t="s">
+        <v>25</v>
+      </c>
+      <c r="D72" s="32" t="s">
+        <v>550</v>
+      </c>
+      <c r="E72" s="32" t="s">
+        <v>551</v>
+      </c>
+      <c r="F72" s="32" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="73" spans="2:6" ht="27">
+      <c r="B73" s="31" t="s">
+        <v>552</v>
+      </c>
+      <c r="C73" s="31" t="s">
+        <v>25</v>
+      </c>
+      <c r="D73" s="32" t="s">
+        <v>553</v>
+      </c>
+      <c r="E73" s="32" t="s">
+        <v>554</v>
+      </c>
+      <c r="F73" s="32" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="74" spans="2:6" ht="27">
+      <c r="B74" s="31" t="s">
+        <v>555</v>
+      </c>
+      <c r="C74" s="31" t="s">
+        <v>25</v>
+      </c>
+      <c r="D74" s="32" t="s">
+        <v>556</v>
+      </c>
+      <c r="E74" s="32" t="s">
+        <v>557</v>
+      </c>
+      <c r="F74" s="32" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="75" spans="2:6" ht="27">
+      <c r="B75" s="31" t="s">
+        <v>558</v>
+      </c>
+      <c r="C75" s="31" t="s">
+        <v>25</v>
+      </c>
+      <c r="D75" s="32" t="s">
+        <v>559</v>
+      </c>
+      <c r="E75" s="32" t="s">
+        <v>560</v>
+      </c>
+      <c r="F75" s="32" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="76" spans="2:6" ht="40.5">
+      <c r="B76" s="31" t="s">
+        <v>561</v>
+      </c>
+      <c r="C76" s="31" t="s">
+        <v>25</v>
+      </c>
+      <c r="D76" s="32" t="s">
+        <v>562</v>
+      </c>
+      <c r="E76" s="32" t="s">
+        <v>563</v>
+      </c>
+      <c r="F76" s="32" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="77" spans="2:6" ht="27">
+      <c r="B77" s="31" t="s">
+        <v>564</v>
+      </c>
+      <c r="C77" s="31" t="s">
+        <v>25</v>
+      </c>
+      <c r="D77" s="32" t="s">
+        <v>565</v>
+      </c>
+      <c r="E77" s="32" t="s">
+        <v>566</v>
+      </c>
+      <c r="F77" s="32" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="78" spans="2:6" ht="27">
+      <c r="B78" s="31" t="s">
+        <v>567</v>
+      </c>
+      <c r="C78" s="31" t="s">
+        <v>25</v>
+      </c>
+      <c r="D78" s="32" t="s">
+        <v>568</v>
+      </c>
+      <c r="E78" s="32" t="s">
+        <v>569</v>
+      </c>
+      <c r="F78" s="32" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="79" spans="2:6" ht="27">
+      <c r="B79" s="31" t="s">
+        <v>570</v>
+      </c>
+      <c r="C79" s="31" t="s">
+        <v>25</v>
+      </c>
+      <c r="D79" s="32" t="s">
+        <v>571</v>
+      </c>
+      <c r="E79" s="32" t="s">
+        <v>572</v>
+      </c>
+      <c r="F79" s="32" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="80" spans="2:6" ht="27">
+      <c r="B80" s="31" t="s">
+        <v>573</v>
+      </c>
+      <c r="C80" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="D80" s="32" t="s">
+        <v>574</v>
+      </c>
+      <c r="E80" s="32" t="s">
+        <v>575</v>
+      </c>
+      <c r="F80" s="32" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="81" spans="2:6" ht="27">
+      <c r="B81" s="31" t="s">
+        <v>576</v>
+      </c>
+      <c r="C81" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="D81" s="32" t="s">
+        <v>577</v>
+      </c>
+      <c r="E81" s="32" t="s">
+        <v>578</v>
+      </c>
+      <c r="F81" s="32" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="82" spans="2:6" ht="27">
+      <c r="B82" s="31" t="s">
+        <v>579</v>
+      </c>
+      <c r="C82" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="D82" s="32" t="s">
+        <v>580</v>
+      </c>
+      <c r="E82" s="32" t="s">
+        <v>581</v>
+      </c>
+      <c r="F82" s="32" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="83" spans="2:6" ht="27">
+      <c r="B83" s="31" t="s">
+        <v>582</v>
+      </c>
+      <c r="C83" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="D83" s="32" t="s">
+        <v>583</v>
+      </c>
+      <c r="E83" s="32" t="s">
+        <v>584</v>
+      </c>
+      <c r="F83" s="32" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="84" spans="2:6" ht="27">
+      <c r="B84" s="31" t="s">
+        <v>585</v>
+      </c>
+      <c r="C84" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="D84" s="32" t="s">
+        <v>586</v>
+      </c>
+      <c r="E84" s="32" t="s">
+        <v>587</v>
+      </c>
+      <c r="F84" s="32" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="85" spans="2:6" ht="27">
+      <c r="B85" s="31" t="s">
+        <v>588</v>
+      </c>
+      <c r="C85" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="D85" s="32" t="s">
+        <v>589</v>
+      </c>
+      <c r="E85" s="32" t="s">
+        <v>590</v>
+      </c>
+      <c r="F85" s="32" t="s">
+        <v>27</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="B5:F5" xr:uid="{CF072275-00C3-4942-9129-BD41CE62AD44}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>